<commit_message>
Remove duplicate nested project directory to fix build path resolution issues
</commit_message>
<xml_diff>
--- a/Final-Price-Template.xlsx
+++ b/Final-Price-Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\diamond_project\ef_rough_diamond_purchase-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BA3585F-CD2C-413B-84F1-6DE481631E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3860770-5E08-4DE6-BD9D-CD63B240FDE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Round" sheetId="1" r:id="rId1"/>
@@ -100,9 +100,6 @@
     <t>0.116-0.158</t>
   </si>
   <si>
-    <t>0.159-0.200</t>
-  </si>
-  <si>
     <t>DEF</t>
   </si>
   <si>
@@ -110,6 +107,9 @@
   </si>
   <si>
     <t>FANCY</t>
+  </si>
+  <si>
+    <t>0.159-0.18</t>
   </si>
 </sst>
 </file>
@@ -328,6 +328,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -344,9 +347,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -645,33 +645,33 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>3</v>
@@ -694,7 +694,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>944.3</v>
@@ -928,20 +928,20 @@
     </row>
     <row r="15" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="12"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>3</v>
@@ -964,7 +964,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17">
         <v>723.8</v>
@@ -1198,20 +1198,20 @@
     </row>
     <row r="26" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>3</v>
@@ -1234,7 +1234,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B28">
         <v>589.4</v>
@@ -1468,20 +1468,20 @@
     </row>
     <row r="37" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="11"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="12"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>3</v>
@@ -1504,7 +1504,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B39">
         <v>583.79999999999995</v>
@@ -1738,20 +1738,20 @@
     </row>
     <row r="48" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
-      <c r="B48" s="9" t="s">
+      <c r="B48" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="11"/>
+      <c r="C48" s="11"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="11"/>
+      <c r="H48" s="12"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>3</v>
@@ -1774,7 +1774,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B50">
         <v>580.29999999999995</v>
@@ -2008,20 +2008,20 @@
     </row>
     <row r="59" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3"/>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C59" s="10"/>
-      <c r="D59" s="10"/>
-      <c r="E59" s="10"/>
-      <c r="F59" s="10"/>
-      <c r="G59" s="10"/>
-      <c r="H59" s="11"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="12"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>3</v>
@@ -2044,7 +2044,7 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B61">
         <v>663.6</v>
@@ -2278,20 +2278,20 @@
     </row>
     <row r="70" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3"/>
-      <c r="B70" s="9" t="s">
+      <c r="B70" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C70" s="10"/>
-      <c r="D70" s="10"/>
-      <c r="E70" s="10"/>
-      <c r="F70" s="10"/>
-      <c r="G70" s="10"/>
-      <c r="H70" s="11"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="12"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C71" s="5" t="s">
         <v>3</v>
@@ -2314,7 +2314,7 @@
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B72">
         <v>747.6</v>
@@ -2548,20 +2548,20 @@
     </row>
     <row r="81" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3"/>
-      <c r="B81" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C81" s="10"/>
-      <c r="D81" s="10"/>
-      <c r="E81" s="10"/>
-      <c r="F81" s="10"/>
-      <c r="G81" s="10"/>
-      <c r="H81" s="11"/>
+      <c r="B81" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C81" s="11"/>
+      <c r="D81" s="11"/>
+      <c r="E81" s="11"/>
+      <c r="F81" s="11"/>
+      <c r="G81" s="11"/>
+      <c r="H81" s="12"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>3</v>
@@ -2584,7 +2584,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B83">
         <v>840</v>
@@ -2818,15 +2818,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B81:H81"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B37:H37"/>
+    <mergeCell ref="B48:H48"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B15:H15"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B70:H70"/>
-    <mergeCell ref="B81:H81"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="B37:H37"/>
-    <mergeCell ref="B48:H48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2841,15 +2841,15 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="8"/>
+      <c r="B1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2863,22 +2863,22 @@
     </row>
     <row r="3" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>3</v>
@@ -2901,27 +2901,27 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="12">
+        <v>24</v>
+      </c>
+      <c r="B5" s="6">
         <v>755.44</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="6">
         <v>603.67999999999995</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="6">
         <v>603.67999999999995</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="6">
         <v>408.24</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="6">
         <v>296.8</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="6">
         <v>185.36</v>
       </c>
     </row>
@@ -2929,25 +2929,25 @@
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="6">
         <v>755.44</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="6">
         <v>346.64</v>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="6">
         <v>259.83999999999997</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="6">
         <v>199.36</v>
       </c>
     </row>
@@ -2955,25 +2955,25 @@
       <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="6">
         <v>519.67999999999995</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="6">
         <v>311.92</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="6">
         <v>234.08</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="6">
         <v>179.2</v>
       </c>
     </row>
@@ -2981,25 +2981,25 @@
       <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="6">
         <v>467.6</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="6">
         <v>467.6</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="6">
         <v>467.6</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="6">
         <v>467.6</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="6">
         <v>280.56</v>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="6">
         <v>154.56</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="6">
         <v>161.28</v>
       </c>
     </row>
@@ -3007,25 +3007,25 @@
       <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="6">
         <v>467.6</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="6">
         <v>467.6</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="6">
         <v>467.6</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="6">
         <v>467.6</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="6">
         <v>280.56</v>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="6">
         <v>154.56</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="6">
         <v>161.28</v>
       </c>
     </row>
@@ -3033,25 +3033,25 @@
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="6">
         <v>421.12</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="6">
         <v>421.12</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="6">
         <v>421.12</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="6">
         <v>421.12</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="6">
         <v>252.56</v>
       </c>
-      <c r="G10" s="12">
+      <c r="G10" s="6">
         <v>189.28</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="6">
         <v>145.04</v>
       </c>
     </row>
@@ -3059,25 +3059,25 @@
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="6">
         <v>378.56</v>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="6">
         <v>378.56</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="6">
         <v>378.56</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="6">
         <v>378.56</v>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="6">
         <v>227.36</v>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="6">
         <v>170.24</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="6">
         <v>130.47999999999999</v>
       </c>
     </row>
@@ -3085,25 +3085,25 @@
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="6">
         <v>378.56</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="6">
         <v>378.56</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="6">
         <v>378.56</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="6">
         <v>378.56</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="6">
         <v>227.36</v>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="6">
         <v>170.24</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="6">
         <v>130.47999999999999</v>
       </c>
     </row>
@@ -3111,44 +3111,44 @@
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="6">
         <v>341.04</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="6">
         <v>341.04</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="6">
         <v>341.04</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="6">
         <v>341.04</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="6">
         <v>204.4</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="6">
         <v>159.04</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="6">
         <v>117.6</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>3</v>
@@ -3171,27 +3171,27 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="12">
+        <v>24</v>
+      </c>
+      <c r="B16" s="6">
         <v>579.04</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="6">
         <v>474.32</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="6">
         <v>474.32</v>
       </c>
-      <c r="E16" s="12">
+      <c r="E16" s="6">
         <v>427.84</v>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="6">
         <v>336</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="6">
         <v>244.72</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="6">
         <v>152.88</v>
       </c>
     </row>
@@ -3199,25 +3199,25 @@
       <c r="A17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="6">
         <v>579.04</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="6">
         <v>427.84</v>
       </c>
-      <c r="D17" s="12">
+      <c r="D17" s="6">
         <v>427.84</v>
       </c>
-      <c r="E17" s="12">
+      <c r="E17" s="6">
         <v>427.84</v>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="6">
         <v>285.04000000000002</v>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="6">
         <v>213.92</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="6">
         <v>164.08</v>
       </c>
     </row>
@@ -3225,25 +3225,25 @@
       <c r="A18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="6">
         <v>427.84</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="6">
         <v>427.84</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="6">
         <v>427.84</v>
       </c>
-      <c r="E18" s="12">
+      <c r="E18" s="6">
         <v>427.84</v>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="6">
         <v>342.16</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="6">
         <v>256.48</v>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3251,25 +3251,25 @@
       <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="6">
         <v>385.28</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="6">
         <v>412.72</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="6">
         <v>346.64</v>
       </c>
-      <c r="E19" s="12">
+      <c r="E19" s="6">
         <v>305.2</v>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="6">
         <v>231.28</v>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="6">
         <v>165.2</v>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="6">
         <v>103.04</v>
       </c>
     </row>
@@ -3277,25 +3277,25 @@
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="6">
         <v>385.28</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="6">
         <v>412.72</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="6">
         <v>346.64</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="6">
         <v>305.2</v>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="6">
         <v>231.28</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="6">
         <v>165.2</v>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="6">
         <v>103.04</v>
       </c>
     </row>
@@ -3303,25 +3303,25 @@
       <c r="A21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="6">
         <v>346.64</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="6">
         <v>288.95999999999998</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="6">
         <v>247.52</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="6">
         <v>206.08</v>
       </c>
-      <c r="F21" s="12">
+      <c r="F21" s="6">
         <v>165.2</v>
       </c>
-      <c r="G21" s="12">
+      <c r="G21" s="6">
         <v>123.76</v>
       </c>
-      <c r="H21" s="12">
+      <c r="H21" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3329,25 +3329,25 @@
       <c r="A22" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="6">
         <v>165.2</v>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="6">
         <v>148.4</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="6">
         <v>140</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="6">
         <v>123.76</v>
       </c>
-      <c r="F22" s="12">
+      <c r="F22" s="6">
         <v>107.52</v>
       </c>
-      <c r="G22" s="12">
-        <v>84</v>
-      </c>
-      <c r="H22" s="12">
+      <c r="G22" s="6">
+        <v>84</v>
+      </c>
+      <c r="H22" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3355,25 +3355,25 @@
       <c r="A23" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="6">
         <v>165.2</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="6">
         <v>148.4</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="6">
         <v>140</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="6">
         <v>123.76</v>
       </c>
-      <c r="F23" s="12">
+      <c r="F23" s="6">
         <v>107.52</v>
       </c>
-      <c r="G23" s="12">
-        <v>84</v>
-      </c>
-      <c r="H23" s="12">
+      <c r="G23" s="6">
+        <v>84</v>
+      </c>
+      <c r="H23" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3381,44 +3381,44 @@
       <c r="A24" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="6">
         <v>123.76</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="6">
         <v>115.36</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="6">
         <v>107.52</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="6">
         <v>99.12</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="6">
         <v>90.72</v>
       </c>
-      <c r="G24" s="12">
-        <v>84</v>
-      </c>
-      <c r="H24" s="12">
+      <c r="G24" s="6">
+        <v>84</v>
+      </c>
+      <c r="H24" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="12"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>3</v>
@@ -3441,27 +3441,27 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B27" s="12">
+        <v>24</v>
+      </c>
+      <c r="B27" s="6">
         <v>471.52</v>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="6">
         <v>396.48</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="6">
         <v>396.48</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="6">
         <v>332.64</v>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="6">
         <v>261.52</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="6">
         <v>189.84</v>
       </c>
-      <c r="H27" s="12">
+      <c r="H27" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3469,25 +3469,25 @@
       <c r="A28" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="6">
         <v>471.52</v>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="6">
         <v>332.64</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="6">
         <v>332.64</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="6">
         <v>332.64</v>
       </c>
-      <c r="F28" s="12">
+      <c r="F28" s="6">
         <v>221.76</v>
       </c>
-      <c r="G28" s="12">
+      <c r="G28" s="6">
         <v>166.32</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3495,25 +3495,25 @@
       <c r="A29" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="6">
         <v>332.64</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="6">
         <v>332.64</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="6">
         <v>332.64</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="6">
         <v>332.64</v>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="6">
         <v>266</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="6">
         <v>199.36</v>
       </c>
-      <c r="H29" s="12">
+      <c r="H29" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3521,25 +3521,25 @@
       <c r="A30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="6">
         <v>299.04000000000002</v>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="6">
         <v>321.44</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="6">
         <v>269.92</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="6">
         <v>237.44</v>
       </c>
-      <c r="F30" s="12">
+      <c r="F30" s="6">
         <v>179.76</v>
       </c>
-      <c r="G30" s="12">
+      <c r="G30" s="6">
         <v>128.24</v>
       </c>
-      <c r="H30" s="12">
+      <c r="H30" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3547,25 +3547,25 @@
       <c r="A31" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="6">
         <v>299.04000000000002</v>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="6">
         <v>321.44</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="6">
         <v>269.92</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="6">
         <v>237.44</v>
       </c>
-      <c r="F31" s="12">
+      <c r="F31" s="6">
         <v>179.76</v>
       </c>
-      <c r="G31" s="12">
+      <c r="G31" s="6">
         <v>128.24</v>
       </c>
-      <c r="H31" s="12">
+      <c r="H31" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3573,25 +3573,25 @@
       <c r="A32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="6">
         <v>269.36</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="6">
         <v>225.12</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="6">
         <v>192.64</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="6">
         <v>160.72</v>
       </c>
-      <c r="F32" s="12">
+      <c r="F32" s="6">
         <v>128.24</v>
       </c>
-      <c r="G32" s="12">
+      <c r="G32" s="6">
         <v>96.32</v>
       </c>
-      <c r="H32" s="12">
+      <c r="H32" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3599,25 +3599,25 @@
       <c r="A33" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="6">
         <v>128.24</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="6">
         <v>115.92</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="6">
         <v>109.2</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E33" s="6">
         <v>96.32</v>
       </c>
-      <c r="F33" s="12">
-        <v>84</v>
-      </c>
-      <c r="G33" s="12">
-        <v>84</v>
-      </c>
-      <c r="H33" s="12">
+      <c r="F33" s="6">
+        <v>84</v>
+      </c>
+      <c r="G33" s="6">
+        <v>84</v>
+      </c>
+      <c r="H33" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3625,25 +3625,25 @@
       <c r="A34" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="6">
         <v>128.24</v>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="6">
         <v>115.92</v>
       </c>
-      <c r="D34" s="12">
+      <c r="D34" s="6">
         <v>109.2</v>
       </c>
-      <c r="E34" s="12">
+      <c r="E34" s="6">
         <v>96.32</v>
       </c>
-      <c r="F34" s="12">
-        <v>84</v>
-      </c>
-      <c r="G34" s="12">
-        <v>84</v>
-      </c>
-      <c r="H34" s="12">
+      <c r="F34" s="6">
+        <v>84</v>
+      </c>
+      <c r="G34" s="6">
+        <v>84</v>
+      </c>
+      <c r="H34" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3651,44 +3651,44 @@
       <c r="A35" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="6">
         <v>96.32</v>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="6">
         <v>90.16</v>
       </c>
-      <c r="D35" s="12">
-        <v>84</v>
-      </c>
-      <c r="E35" s="12">
-        <v>84</v>
-      </c>
-      <c r="F35" s="12">
-        <v>84</v>
-      </c>
-      <c r="G35" s="12">
-        <v>84</v>
-      </c>
-      <c r="H35" s="12">
+      <c r="D35" s="6">
+        <v>84</v>
+      </c>
+      <c r="E35" s="6">
+        <v>84</v>
+      </c>
+      <c r="F35" s="6">
+        <v>84</v>
+      </c>
+      <c r="G35" s="6">
+        <v>84</v>
+      </c>
+      <c r="H35" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="12"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>3</v>
@@ -3711,27 +3711,27 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B38" s="12">
+        <v>24</v>
+      </c>
+      <c r="B38" s="6">
         <v>467.04</v>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="6">
         <v>395.92</v>
       </c>
-      <c r="D38" s="12">
+      <c r="D38" s="6">
         <v>395.92</v>
       </c>
-      <c r="E38" s="12">
+      <c r="E38" s="6">
         <v>322.56</v>
       </c>
-      <c r="F38" s="12">
+      <c r="F38" s="6">
         <v>253.12</v>
       </c>
-      <c r="G38" s="12">
+      <c r="G38" s="6">
         <v>184.24</v>
       </c>
-      <c r="H38" s="12">
+      <c r="H38" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3739,25 +3739,25 @@
       <c r="A39" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="6">
         <v>467.04</v>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="6">
         <v>322.56</v>
       </c>
-      <c r="D39" s="12">
+      <c r="D39" s="6">
         <v>322.56</v>
       </c>
-      <c r="E39" s="12">
+      <c r="E39" s="6">
         <v>322.56</v>
       </c>
-      <c r="F39" s="12">
+      <c r="F39" s="6">
         <v>215.04</v>
       </c>
-      <c r="G39" s="12">
+      <c r="G39" s="6">
         <v>161.28</v>
       </c>
-      <c r="H39" s="12">
+      <c r="H39" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3765,25 +3765,25 @@
       <c r="A40" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="6">
         <v>322.56</v>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="6">
         <v>322.56</v>
       </c>
-      <c r="D40" s="12">
+      <c r="D40" s="6">
         <v>322.56</v>
       </c>
-      <c r="E40" s="12">
+      <c r="E40" s="6">
         <v>322.56</v>
       </c>
-      <c r="F40" s="12">
+      <c r="F40" s="6">
         <v>258.16000000000003</v>
       </c>
-      <c r="G40" s="12">
+      <c r="G40" s="6">
         <v>193.76</v>
       </c>
-      <c r="H40" s="12">
+      <c r="H40" s="6">
         <v>140</v>
       </c>
     </row>
@@ -3791,25 +3791,25 @@
       <c r="A41" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="6">
         <v>290.08</v>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="6">
         <v>311.36</v>
       </c>
-      <c r="D41" s="12">
+      <c r="D41" s="6">
         <v>261.52</v>
       </c>
-      <c r="E41" s="12">
+      <c r="E41" s="6">
         <v>230.16</v>
       </c>
-      <c r="F41" s="12">
+      <c r="F41" s="6">
         <v>174.16</v>
       </c>
-      <c r="G41" s="12">
+      <c r="G41" s="6">
         <v>124.32</v>
       </c>
-      <c r="H41" s="12">
+      <c r="H41" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3817,25 +3817,25 @@
       <c r="A42" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="6">
         <v>290.08</v>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="6">
         <v>311.36</v>
       </c>
-      <c r="D42" s="12">
+      <c r="D42" s="6">
         <v>261.52</v>
       </c>
-      <c r="E42" s="12">
+      <c r="E42" s="6">
         <v>230.16</v>
       </c>
-      <c r="F42" s="12">
+      <c r="F42" s="6">
         <v>174.16</v>
       </c>
-      <c r="G42" s="12">
+      <c r="G42" s="6">
         <v>124.32</v>
       </c>
-      <c r="H42" s="12">
+      <c r="H42" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3843,25 +3843,25 @@
       <c r="A43" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="6">
         <v>260.95999999999998</v>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="6">
         <v>217.84</v>
       </c>
-      <c r="D43" s="12">
+      <c r="D43" s="6">
         <v>186.48</v>
       </c>
-      <c r="E43" s="12">
+      <c r="E43" s="6">
         <v>155.68</v>
       </c>
-      <c r="F43" s="12">
+      <c r="F43" s="6">
         <v>124.32</v>
       </c>
-      <c r="G43" s="12">
+      <c r="G43" s="6">
         <v>93.52</v>
       </c>
-      <c r="H43" s="12">
+      <c r="H43" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3869,25 +3869,25 @@
       <c r="A44" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="6">
         <v>124.32</v>
       </c>
-      <c r="C44" s="12">
+      <c r="C44" s="6">
         <v>112</v>
       </c>
-      <c r="D44" s="12">
+      <c r="D44" s="6">
         <v>105.84</v>
       </c>
-      <c r="E44" s="12">
+      <c r="E44" s="6">
         <v>93.52</v>
       </c>
-      <c r="F44" s="12">
-        <v>84</v>
-      </c>
-      <c r="G44" s="12">
-        <v>84</v>
-      </c>
-      <c r="H44" s="12">
+      <c r="F44" s="6">
+        <v>84</v>
+      </c>
+      <c r="G44" s="6">
+        <v>84</v>
+      </c>
+      <c r="H44" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3895,25 +3895,25 @@
       <c r="A45" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="6">
         <v>124.32</v>
       </c>
-      <c r="C45" s="12">
+      <c r="C45" s="6">
         <v>112</v>
       </c>
-      <c r="D45" s="12">
+      <c r="D45" s="6">
         <v>105.84</v>
       </c>
-      <c r="E45" s="12">
+      <c r="E45" s="6">
         <v>93.52</v>
       </c>
-      <c r="F45" s="12">
-        <v>84</v>
-      </c>
-      <c r="G45" s="12">
-        <v>84</v>
-      </c>
-      <c r="H45" s="12">
+      <c r="F45" s="6">
+        <v>84</v>
+      </c>
+      <c r="G45" s="6">
+        <v>84</v>
+      </c>
+      <c r="H45" s="6">
         <v>84</v>
       </c>
     </row>
@@ -3921,44 +3921,44 @@
       <c r="A46" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="6">
         <v>93.52</v>
       </c>
-      <c r="C46" s="12">
+      <c r="C46" s="6">
         <v>87.36</v>
       </c>
-      <c r="D46" s="12">
-        <v>84</v>
-      </c>
-      <c r="E46" s="12">
-        <v>84</v>
-      </c>
-      <c r="F46" s="12">
-        <v>84</v>
-      </c>
-      <c r="G46" s="12">
-        <v>84</v>
-      </c>
-      <c r="H46" s="12">
+      <c r="D46" s="6">
+        <v>84</v>
+      </c>
+      <c r="E46" s="6">
+        <v>84</v>
+      </c>
+      <c r="F46" s="6">
+        <v>84</v>
+      </c>
+      <c r="G46" s="6">
+        <v>84</v>
+      </c>
+      <c r="H46" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
-      <c r="B47" s="9" t="s">
+      <c r="B47" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="11"/>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="11"/>
+      <c r="H47" s="12"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>3</v>
@@ -3981,27 +3981,27 @@
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B49" s="12">
+        <v>24</v>
+      </c>
+      <c r="B49" s="6">
         <v>464.24</v>
       </c>
-      <c r="C49" s="12">
+      <c r="C49" s="6">
         <v>408.8</v>
       </c>
-      <c r="D49" s="12">
+      <c r="D49" s="6">
         <v>408.8</v>
       </c>
-      <c r="E49" s="12">
+      <c r="E49" s="6">
         <v>330.4</v>
       </c>
-      <c r="F49" s="12">
+      <c r="F49" s="6">
         <v>259.83999999999997</v>
       </c>
-      <c r="G49" s="12">
+      <c r="G49" s="6">
         <v>188.72</v>
       </c>
-      <c r="H49" s="12">
+      <c r="H49" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4009,25 +4009,25 @@
       <c r="A50" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="6">
         <v>464.24</v>
       </c>
-      <c r="C50" s="12">
+      <c r="C50" s="6">
         <v>330.4</v>
       </c>
-      <c r="D50" s="12">
+      <c r="D50" s="6">
         <v>330.4</v>
       </c>
-      <c r="E50" s="12">
+      <c r="E50" s="6">
         <v>330.4</v>
       </c>
-      <c r="F50" s="12">
+      <c r="F50" s="6">
         <v>220.64</v>
       </c>
-      <c r="G50" s="12">
+      <c r="G50" s="6">
         <v>165.2</v>
       </c>
-      <c r="H50" s="12">
+      <c r="H50" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4035,25 +4035,25 @@
       <c r="A51" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="6">
         <v>330.4</v>
       </c>
-      <c r="C51" s="12">
+      <c r="C51" s="6">
         <v>330.4</v>
       </c>
-      <c r="D51" s="12">
+      <c r="D51" s="6">
         <v>330.4</v>
       </c>
-      <c r="E51" s="12">
+      <c r="E51" s="6">
         <v>330.4</v>
       </c>
-      <c r="F51" s="12">
+      <c r="F51" s="6">
         <v>264.32</v>
       </c>
-      <c r="G51" s="12">
+      <c r="G51" s="6">
         <v>198.24</v>
       </c>
-      <c r="H51" s="12">
+      <c r="H51" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4061,25 +4061,25 @@
       <c r="A52" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="12">
+      <c r="B52" s="6">
         <v>297.36</v>
       </c>
-      <c r="C52" s="12">
+      <c r="C52" s="6">
         <v>318.64</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D52" s="6">
         <v>267.68</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E52" s="6">
         <v>235.76</v>
       </c>
-      <c r="F52" s="12">
+      <c r="F52" s="6">
         <v>178.08</v>
       </c>
-      <c r="G52" s="12">
+      <c r="G52" s="6">
         <v>127.12</v>
       </c>
-      <c r="H52" s="12">
+      <c r="H52" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4087,25 +4087,25 @@
       <c r="A53" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="6">
         <v>297.36</v>
       </c>
-      <c r="C53" s="12">
+      <c r="C53" s="6">
         <v>318.64</v>
       </c>
-      <c r="D53" s="12">
+      <c r="D53" s="6">
         <v>267.68</v>
       </c>
-      <c r="E53" s="12">
+      <c r="E53" s="6">
         <v>235.76</v>
       </c>
-      <c r="F53" s="12">
+      <c r="F53" s="6">
         <v>178.08</v>
       </c>
-      <c r="G53" s="12">
+      <c r="G53" s="6">
         <v>127.12</v>
       </c>
-      <c r="H53" s="12">
+      <c r="H53" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4113,25 +4113,25 @@
       <c r="A54" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="6">
         <v>267.68</v>
       </c>
-      <c r="C54" s="12">
+      <c r="C54" s="6">
         <v>222.88</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D54" s="6">
         <v>190.96</v>
       </c>
-      <c r="E54" s="12">
+      <c r="E54" s="6">
         <v>159.04</v>
       </c>
-      <c r="F54" s="12">
+      <c r="F54" s="6">
         <v>127.12</v>
       </c>
-      <c r="G54" s="12">
+      <c r="G54" s="6">
         <v>95.76</v>
       </c>
-      <c r="H54" s="12">
+      <c r="H54" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4139,25 +4139,25 @@
       <c r="A55" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="6">
         <v>127.12</v>
       </c>
-      <c r="C55" s="12">
+      <c r="C55" s="6">
         <v>114.8</v>
       </c>
-      <c r="D55" s="12">
+      <c r="D55" s="6">
         <v>108.08</v>
       </c>
-      <c r="E55" s="12">
+      <c r="E55" s="6">
         <v>95.76</v>
       </c>
-      <c r="F55" s="12">
-        <v>84</v>
-      </c>
-      <c r="G55" s="12">
-        <v>84</v>
-      </c>
-      <c r="H55" s="12">
+      <c r="F55" s="6">
+        <v>84</v>
+      </c>
+      <c r="G55" s="6">
+        <v>84</v>
+      </c>
+      <c r="H55" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4165,25 +4165,25 @@
       <c r="A56" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="6">
         <v>127.12</v>
       </c>
-      <c r="C56" s="12">
+      <c r="C56" s="6">
         <v>114.8</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D56" s="6">
         <v>108.08</v>
       </c>
-      <c r="E56" s="12">
+      <c r="E56" s="6">
         <v>95.76</v>
       </c>
-      <c r="F56" s="12">
-        <v>84</v>
-      </c>
-      <c r="G56" s="12">
-        <v>84</v>
-      </c>
-      <c r="H56" s="12">
+      <c r="F56" s="6">
+        <v>84</v>
+      </c>
+      <c r="G56" s="6">
+        <v>84</v>
+      </c>
+      <c r="H56" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4191,44 +4191,44 @@
       <c r="A57" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B57" s="12">
+      <c r="B57" s="6">
         <v>95.76</v>
       </c>
-      <c r="C57" s="12">
+      <c r="C57" s="6">
         <v>89.04</v>
       </c>
-      <c r="D57" s="12">
-        <v>84</v>
-      </c>
-      <c r="E57" s="12">
-        <v>84</v>
-      </c>
-      <c r="F57" s="12">
-        <v>84</v>
-      </c>
-      <c r="G57" s="12">
-        <v>84</v>
-      </c>
-      <c r="H57" s="12">
+      <c r="D57" s="6">
+        <v>84</v>
+      </c>
+      <c r="E57" s="6">
+        <v>84</v>
+      </c>
+      <c r="F57" s="6">
+        <v>84</v>
+      </c>
+      <c r="G57" s="6">
+        <v>84</v>
+      </c>
+      <c r="H57" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
-      <c r="B58" s="9" t="s">
+      <c r="B58" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="12"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>3</v>
@@ -4251,27 +4251,27 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B60" s="12">
+        <v>24</v>
+      </c>
+      <c r="B60" s="6">
         <v>530.88</v>
       </c>
-      <c r="C60" s="12">
+      <c r="C60" s="6">
         <v>478.8</v>
       </c>
-      <c r="D60" s="12">
+      <c r="D60" s="6">
         <v>478.8</v>
       </c>
-      <c r="E60" s="12">
+      <c r="E60" s="6">
         <v>391.44</v>
       </c>
-      <c r="F60" s="12">
+      <c r="F60" s="6">
         <v>307.44</v>
       </c>
-      <c r="G60" s="12">
+      <c r="G60" s="6">
         <v>223.44</v>
       </c>
-      <c r="H60" s="12">
+      <c r="H60" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4279,25 +4279,25 @@
       <c r="A61" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B61" s="12">
+      <c r="B61" s="6">
         <v>530.88</v>
       </c>
-      <c r="C61" s="12">
+      <c r="C61" s="6">
         <v>391.44</v>
       </c>
-      <c r="D61" s="12">
+      <c r="D61" s="6">
         <v>391.44</v>
       </c>
-      <c r="E61" s="12">
+      <c r="E61" s="6">
         <v>391.44</v>
       </c>
-      <c r="F61" s="12">
+      <c r="F61" s="6">
         <v>260.95999999999998</v>
       </c>
-      <c r="G61" s="12">
+      <c r="G61" s="6">
         <v>196</v>
       </c>
-      <c r="H61" s="12">
+      <c r="H61" s="6">
         <v>150.08000000000001</v>
       </c>
     </row>
@@ -4305,25 +4305,25 @@
       <c r="A62" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B62" s="12">
+      <c r="B62" s="6">
         <v>391.44</v>
       </c>
-      <c r="C62" s="12">
+      <c r="C62" s="6">
         <v>391.44</v>
       </c>
-      <c r="D62" s="12">
+      <c r="D62" s="6">
         <v>391.44</v>
       </c>
-      <c r="E62" s="12">
+      <c r="E62" s="6">
         <v>391.44</v>
       </c>
-      <c r="F62" s="12">
+      <c r="F62" s="6">
         <v>313.04000000000002</v>
       </c>
-      <c r="G62" s="12">
+      <c r="G62" s="6">
         <v>234.64</v>
       </c>
-      <c r="H62" s="12">
+      <c r="H62" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4331,25 +4331,25 @@
       <c r="A63" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B63" s="12">
+      <c r="B63" s="6">
         <v>352.24</v>
       </c>
-      <c r="C63" s="12">
+      <c r="C63" s="6">
         <v>377.44</v>
       </c>
-      <c r="D63" s="12">
+      <c r="D63" s="6">
         <v>316.95999999999998</v>
       </c>
-      <c r="E63" s="12">
+      <c r="E63" s="6">
         <v>279.44</v>
       </c>
-      <c r="F63" s="12">
+      <c r="F63" s="6">
         <v>211.12</v>
       </c>
-      <c r="G63" s="12">
+      <c r="G63" s="6">
         <v>151.19999999999999</v>
       </c>
-      <c r="H63" s="12">
+      <c r="H63" s="6">
         <v>94.08</v>
       </c>
     </row>
@@ -4357,25 +4357,25 @@
       <c r="A64" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B64" s="12">
+      <c r="B64" s="6">
         <v>352.24</v>
       </c>
-      <c r="C64" s="12">
+      <c r="C64" s="6">
         <v>377.44</v>
       </c>
-      <c r="D64" s="12">
+      <c r="D64" s="6">
         <v>316.95999999999998</v>
       </c>
-      <c r="E64" s="12">
+      <c r="E64" s="6">
         <v>279.44</v>
       </c>
-      <c r="F64" s="12">
+      <c r="F64" s="6">
         <v>211.12</v>
       </c>
-      <c r="G64" s="12">
+      <c r="G64" s="6">
         <v>151.19999999999999</v>
       </c>
-      <c r="H64" s="12">
+      <c r="H64" s="6">
         <v>94.08</v>
       </c>
     </row>
@@ -4383,25 +4383,25 @@
       <c r="A65" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B65" s="12">
+      <c r="B65" s="6">
         <v>316.95999999999998</v>
       </c>
-      <c r="C65" s="12">
+      <c r="C65" s="6">
         <v>264.32</v>
       </c>
-      <c r="D65" s="12">
+      <c r="D65" s="6">
         <v>226.24</v>
       </c>
-      <c r="E65" s="12">
+      <c r="E65" s="6">
         <v>188.72</v>
       </c>
-      <c r="F65" s="12">
+      <c r="F65" s="6">
         <v>151.19999999999999</v>
       </c>
-      <c r="G65" s="12">
+      <c r="G65" s="6">
         <v>113.12</v>
       </c>
-      <c r="H65" s="12">
+      <c r="H65" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4409,25 +4409,25 @@
       <c r="A66" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B66" s="12">
+      <c r="B66" s="6">
         <v>151.19999999999999</v>
       </c>
-      <c r="C66" s="12">
+      <c r="C66" s="6">
         <v>136.08000000000001</v>
       </c>
-      <c r="D66" s="12">
+      <c r="D66" s="6">
         <v>128.24</v>
       </c>
-      <c r="E66" s="12">
+      <c r="E66" s="6">
         <v>113.12</v>
       </c>
-      <c r="F66" s="12">
+      <c r="F66" s="6">
         <v>98</v>
       </c>
-      <c r="G66" s="12">
-        <v>84</v>
-      </c>
-      <c r="H66" s="12">
+      <c r="G66" s="6">
+        <v>84</v>
+      </c>
+      <c r="H66" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4435,25 +4435,25 @@
       <c r="A67" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B67" s="12">
+      <c r="B67" s="6">
         <v>151.19999999999999</v>
       </c>
-      <c r="C67" s="12">
+      <c r="C67" s="6">
         <v>136.08000000000001</v>
       </c>
-      <c r="D67" s="12">
+      <c r="D67" s="6">
         <v>128.24</v>
       </c>
-      <c r="E67" s="12">
+      <c r="E67" s="6">
         <v>113.12</v>
       </c>
-      <c r="F67" s="12">
+      <c r="F67" s="6">
         <v>98</v>
       </c>
-      <c r="G67" s="12">
-        <v>84</v>
-      </c>
-      <c r="H67" s="12">
+      <c r="G67" s="6">
+        <v>84</v>
+      </c>
+      <c r="H67" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4461,44 +4461,44 @@
       <c r="A68" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B68" s="12">
+      <c r="B68" s="6">
         <v>113.12</v>
       </c>
-      <c r="C68" s="12">
+      <c r="C68" s="6">
         <v>105.84</v>
       </c>
-      <c r="D68" s="12">
+      <c r="D68" s="6">
         <v>98</v>
       </c>
-      <c r="E68" s="12">
+      <c r="E68" s="6">
         <v>90.72</v>
       </c>
-      <c r="F68" s="12">
-        <v>84</v>
-      </c>
-      <c r="G68" s="12">
-        <v>84</v>
-      </c>
-      <c r="H68" s="12">
+      <c r="F68" s="6">
+        <v>84</v>
+      </c>
+      <c r="G68" s="6">
+        <v>84</v>
+      </c>
+      <c r="H68" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3"/>
-      <c r="B69" s="9" t="s">
+      <c r="B69" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C69" s="10"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
-      <c r="G69" s="10"/>
-      <c r="H69" s="11"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="12"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
       <c r="B70" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>3</v>
@@ -4521,27 +4521,27 @@
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B71" s="12">
+        <v>24</v>
+      </c>
+      <c r="B71" s="6">
         <v>598.08000000000004</v>
       </c>
-      <c r="C71" s="12">
+      <c r="C71" s="6">
         <v>539.28</v>
       </c>
-      <c r="D71" s="12">
+      <c r="D71" s="6">
         <v>539.28</v>
       </c>
-      <c r="E71" s="12">
+      <c r="E71" s="6">
         <v>443.52</v>
       </c>
-      <c r="F71" s="12">
+      <c r="F71" s="6">
         <v>348.88</v>
       </c>
-      <c r="G71" s="12">
+      <c r="G71" s="6">
         <v>253.68</v>
       </c>
-      <c r="H71" s="12">
+      <c r="H71" s="6">
         <v>158.47999999999999</v>
       </c>
     </row>
@@ -4549,25 +4549,25 @@
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B72" s="12">
+      <c r="B72" s="6">
         <v>598.08000000000004</v>
       </c>
-      <c r="C72" s="12">
+      <c r="C72" s="6">
         <v>443.52</v>
       </c>
-      <c r="D72" s="12">
+      <c r="D72" s="6">
         <v>443.52</v>
       </c>
-      <c r="E72" s="12">
+      <c r="E72" s="6">
         <v>443.52</v>
       </c>
-      <c r="F72" s="12">
+      <c r="F72" s="6">
         <v>295.68</v>
       </c>
-      <c r="G72" s="12">
+      <c r="G72" s="6">
         <v>221.76</v>
       </c>
-      <c r="H72" s="12">
+      <c r="H72" s="6">
         <v>170.24</v>
       </c>
     </row>
@@ -4575,25 +4575,25 @@
       <c r="A73" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B73" s="12">
+      <c r="B73" s="6">
         <v>443.52</v>
       </c>
-      <c r="C73" s="12">
+      <c r="C73" s="6">
         <v>443.52</v>
       </c>
-      <c r="D73" s="12">
+      <c r="D73" s="6">
         <v>443.52</v>
       </c>
-      <c r="E73" s="12">
+      <c r="E73" s="6">
         <v>443.52</v>
       </c>
-      <c r="F73" s="12">
+      <c r="F73" s="6">
         <v>355.04</v>
       </c>
-      <c r="G73" s="12">
+      <c r="G73" s="6">
         <v>266</v>
       </c>
-      <c r="H73" s="12">
+      <c r="H73" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4601,25 +4601,25 @@
       <c r="A74" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B74" s="12">
+      <c r="B74" s="6">
         <v>399.28</v>
       </c>
-      <c r="C74" s="12">
+      <c r="C74" s="6">
         <v>428.4</v>
       </c>
-      <c r="D74" s="12">
+      <c r="D74" s="6">
         <v>359.52</v>
       </c>
-      <c r="E74" s="12">
+      <c r="E74" s="6">
         <v>316.95999999999998</v>
       </c>
-      <c r="F74" s="12">
+      <c r="F74" s="6">
         <v>239.68</v>
       </c>
-      <c r="G74" s="12">
+      <c r="G74" s="6">
         <v>171.36</v>
       </c>
-      <c r="H74" s="12">
+      <c r="H74" s="6">
         <v>106.96</v>
       </c>
     </row>
@@ -4627,25 +4627,25 @@
       <c r="A75" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="12">
+      <c r="B75" s="6">
         <v>399.28</v>
       </c>
-      <c r="C75" s="12">
+      <c r="C75" s="6">
         <v>428.4</v>
       </c>
-      <c r="D75" s="12">
+      <c r="D75" s="6">
         <v>359.52</v>
       </c>
-      <c r="E75" s="12">
+      <c r="E75" s="6">
         <v>316.95999999999998</v>
       </c>
-      <c r="F75" s="12">
+      <c r="F75" s="6">
         <v>239.68</v>
       </c>
-      <c r="G75" s="12">
+      <c r="G75" s="6">
         <v>171.36</v>
       </c>
-      <c r="H75" s="12">
+      <c r="H75" s="6">
         <v>106.96</v>
       </c>
     </row>
@@ -4653,25 +4653,25 @@
       <c r="A76" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B76" s="12">
+      <c r="B76" s="6">
         <v>359.52</v>
       </c>
-      <c r="C76" s="12">
+      <c r="C76" s="6">
         <v>299.60000000000002</v>
       </c>
-      <c r="D76" s="12">
+      <c r="D76" s="6">
         <v>257.04000000000002</v>
       </c>
-      <c r="E76" s="12">
+      <c r="E76" s="6">
         <v>213.92</v>
       </c>
-      <c r="F76" s="12">
+      <c r="F76" s="6">
         <v>171.36</v>
       </c>
-      <c r="G76" s="12">
+      <c r="G76" s="6">
         <v>128.24</v>
       </c>
-      <c r="H76" s="12">
+      <c r="H76" s="6">
         <v>85.68</v>
       </c>
     </row>
@@ -4679,25 +4679,25 @@
       <c r="A77" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B77" s="12">
+      <c r="B77" s="6">
         <v>171.36</v>
       </c>
-      <c r="C77" s="12">
+      <c r="C77" s="6">
         <v>154</v>
       </c>
-      <c r="D77" s="12">
+      <c r="D77" s="6">
         <v>145.6</v>
       </c>
-      <c r="E77" s="12">
+      <c r="E77" s="6">
         <v>128.24</v>
       </c>
-      <c r="F77" s="12">
+      <c r="F77" s="6">
         <v>111.44</v>
       </c>
-      <c r="G77" s="12">
+      <c r="G77" s="6">
         <v>85.68</v>
       </c>
-      <c r="H77" s="12">
+      <c r="H77" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4705,25 +4705,25 @@
       <c r="A78" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B78" s="12">
+      <c r="B78" s="6">
         <v>171.36</v>
       </c>
-      <c r="C78" s="12">
+      <c r="C78" s="6">
         <v>154</v>
       </c>
-      <c r="D78" s="12">
+      <c r="D78" s="6">
         <v>145.6</v>
       </c>
-      <c r="E78" s="12">
+      <c r="E78" s="6">
         <v>128.24</v>
       </c>
-      <c r="F78" s="12">
+      <c r="F78" s="6">
         <v>111.44</v>
       </c>
-      <c r="G78" s="12">
+      <c r="G78" s="6">
         <v>85.68</v>
       </c>
-      <c r="H78" s="12">
+      <c r="H78" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4731,44 +4731,44 @@
       <c r="A79" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B79" s="12">
+      <c r="B79" s="6">
         <v>128.24</v>
       </c>
-      <c r="C79" s="12">
+      <c r="C79" s="6">
         <v>119.84</v>
       </c>
-      <c r="D79" s="12">
+      <c r="D79" s="6">
         <v>111.44</v>
       </c>
-      <c r="E79" s="12">
+      <c r="E79" s="6">
         <v>103.04</v>
       </c>
-      <c r="F79" s="12">
+      <c r="F79" s="6">
         <v>94.08</v>
       </c>
-      <c r="G79" s="12">
+      <c r="G79" s="6">
         <v>85.68</v>
       </c>
-      <c r="H79" s="12">
+      <c r="H79" s="6">
         <v>84</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3"/>
-      <c r="B80" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C80" s="10"/>
-      <c r="D80" s="10"/>
-      <c r="E80" s="10"/>
-      <c r="F80" s="10"/>
-      <c r="G80" s="10"/>
-      <c r="H80" s="11"/>
+      <c r="B80" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80" s="11"/>
+      <c r="D80" s="11"/>
+      <c r="E80" s="11"/>
+      <c r="F80" s="11"/>
+      <c r="G80" s="11"/>
+      <c r="H80" s="12"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C81" s="5" t="s">
         <v>3</v>
@@ -4791,27 +4791,27 @@
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B82" s="12">
+        <v>24</v>
+      </c>
+      <c r="B82" s="6">
         <v>672</v>
       </c>
-      <c r="C82" s="12">
+      <c r="C82" s="6">
         <v>616</v>
       </c>
-      <c r="D82" s="12">
+      <c r="D82" s="6">
         <v>504</v>
       </c>
-      <c r="E82" s="12">
+      <c r="E82" s="6">
         <v>392</v>
       </c>
-      <c r="F82" s="12">
+      <c r="F82" s="6">
         <v>308</v>
       </c>
-      <c r="G82" s="12">
+      <c r="G82" s="6">
         <v>224</v>
       </c>
-      <c r="H82" s="12">
+      <c r="H82" s="6">
         <v>140</v>
       </c>
     </row>
@@ -4819,25 +4819,25 @@
       <c r="A83" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B83" s="12">
+      <c r="B83" s="6">
         <v>560</v>
       </c>
-      <c r="C83" s="12">
+      <c r="C83" s="6">
         <v>448</v>
       </c>
-      <c r="D83" s="12">
+      <c r="D83" s="6">
         <v>392</v>
       </c>
-      <c r="E83" s="12">
+      <c r="E83" s="6">
         <v>336</v>
       </c>
-      <c r="F83" s="12">
+      <c r="F83" s="6">
         <v>224</v>
       </c>
-      <c r="G83" s="12">
+      <c r="G83" s="6">
         <v>168</v>
       </c>
-      <c r="H83" s="12">
+      <c r="H83" s="6">
         <v>128.80000000000001</v>
       </c>
     </row>
@@ -4845,25 +4845,25 @@
       <c r="A84" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B84" s="12">
+      <c r="B84" s="6">
         <v>448</v>
       </c>
-      <c r="C84" s="12">
+      <c r="C84" s="6">
         <v>392</v>
       </c>
-      <c r="D84" s="12">
+      <c r="D84" s="6">
         <v>336</v>
       </c>
-      <c r="E84" s="12">
+      <c r="E84" s="6">
         <v>280</v>
       </c>
-      <c r="F84" s="12">
+      <c r="F84" s="6">
         <v>224</v>
       </c>
-      <c r="G84" s="12">
+      <c r="G84" s="6">
         <v>168</v>
       </c>
-      <c r="H84" s="12">
+      <c r="H84" s="6">
         <v>84</v>
       </c>
     </row>
@@ -4871,25 +4871,25 @@
       <c r="A85" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B85" s="12">
+      <c r="B85" s="6">
         <v>336</v>
       </c>
-      <c r="C85" s="12">
+      <c r="C85" s="6">
         <v>280</v>
       </c>
-      <c r="D85" s="12">
+      <c r="D85" s="6">
         <v>235.2</v>
       </c>
-      <c r="E85" s="12">
+      <c r="E85" s="6">
         <v>207.2</v>
       </c>
-      <c r="F85" s="12">
+      <c r="F85" s="6">
         <v>156.80000000000001</v>
       </c>
-      <c r="G85" s="12">
+      <c r="G85" s="6">
         <v>112</v>
       </c>
-      <c r="H85" s="12">
+      <c r="H85" s="6">
         <v>70</v>
       </c>
     </row>
@@ -4897,25 +4897,25 @@
       <c r="A86" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B86" s="12">
+      <c r="B86" s="6">
         <v>336</v>
       </c>
-      <c r="C86" s="12">
+      <c r="C86" s="6">
         <v>280</v>
       </c>
-      <c r="D86" s="12">
+      <c r="D86" s="6">
         <v>235.2</v>
       </c>
-      <c r="E86" s="12">
+      <c r="E86" s="6">
         <v>207.2</v>
       </c>
-      <c r="F86" s="12">
+      <c r="F86" s="6">
         <v>156.80000000000001</v>
       </c>
-      <c r="G86" s="12">
+      <c r="G86" s="6">
         <v>112</v>
       </c>
-      <c r="H86" s="12">
+      <c r="H86" s="6">
         <v>70</v>
       </c>
     </row>
@@ -4923,25 +4923,25 @@
       <c r="A87" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B87" s="12">
+      <c r="B87" s="6">
         <v>224</v>
       </c>
-      <c r="C87" s="12">
+      <c r="C87" s="6">
         <v>196</v>
       </c>
-      <c r="D87" s="12">
+      <c r="D87" s="6">
         <v>168</v>
       </c>
-      <c r="E87" s="12">
+      <c r="E87" s="6">
         <v>140</v>
       </c>
-      <c r="F87" s="12">
+      <c r="F87" s="6">
         <v>112</v>
       </c>
-      <c r="G87" s="12">
-        <v>84</v>
-      </c>
-      <c r="H87" s="12">
+      <c r="G87" s="6">
+        <v>84</v>
+      </c>
+      <c r="H87" s="6">
         <v>56</v>
       </c>
     </row>
@@ -4949,25 +4949,25 @@
       <c r="A88" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B88" s="12">
+      <c r="B88" s="6">
         <v>112</v>
       </c>
-      <c r="C88" s="12">
+      <c r="C88" s="6">
         <v>100.8</v>
       </c>
-      <c r="D88" s="12">
+      <c r="D88" s="6">
         <v>95.2</v>
       </c>
-      <c r="E88" s="12">
-        <v>84</v>
-      </c>
-      <c r="F88" s="12">
+      <c r="E88" s="6">
+        <v>84</v>
+      </c>
+      <c r="F88" s="6">
         <v>72.8</v>
       </c>
-      <c r="G88" s="12">
+      <c r="G88" s="6">
         <v>56</v>
       </c>
-      <c r="H88" s="12">
+      <c r="H88" s="6">
         <v>50.4</v>
       </c>
     </row>
@@ -4975,25 +4975,25 @@
       <c r="A89" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B89" s="12">
+      <c r="B89" s="6">
         <v>112</v>
       </c>
-      <c r="C89" s="12">
+      <c r="C89" s="6">
         <v>100.8</v>
       </c>
-      <c r="D89" s="12">
+      <c r="D89" s="6">
         <v>95.2</v>
       </c>
-      <c r="E89" s="12">
-        <v>84</v>
-      </c>
-      <c r="F89" s="12">
+      <c r="E89" s="6">
+        <v>84</v>
+      </c>
+      <c r="F89" s="6">
         <v>72.8</v>
       </c>
-      <c r="G89" s="12">
+      <c r="G89" s="6">
         <v>56</v>
       </c>
-      <c r="H89" s="12">
+      <c r="H89" s="6">
         <v>50.4</v>
       </c>
     </row>
@@ -5001,25 +5001,25 @@
       <c r="A90" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B90" s="12">
-        <v>84</v>
-      </c>
-      <c r="C90" s="12">
+      <c r="B90" s="6">
+        <v>84</v>
+      </c>
+      <c r="C90" s="6">
         <v>78.400000000000006</v>
       </c>
-      <c r="D90" s="12">
+      <c r="D90" s="6">
         <v>72.8</v>
       </c>
-      <c r="E90" s="12">
+      <c r="E90" s="6">
         <v>67.2</v>
       </c>
-      <c r="F90" s="12">
+      <c r="F90" s="6">
         <v>61.6</v>
       </c>
-      <c r="G90" s="12">
+      <c r="G90" s="6">
         <v>56</v>
       </c>
-      <c r="H90" s="12">
+      <c r="H90" s="6">
         <v>44.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CHECKPOINT - Before implementing price use previous category feature
</commit_message>
<xml_diff>
--- a/Final-Price-Template.xlsx
+++ b/Final-Price-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\diamond_project\ef_rough_diamond_purchase-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3860770-5E08-4DE6-BD9D-CD63B240FDE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2584A8-D19A-4F54-943B-F4B0C8D007CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="36">
   <si>
     <t>SHAPE</t>
   </si>
@@ -110,6 +110,30 @@
   </si>
   <si>
     <t>0.159-0.18</t>
+  </si>
+  <si>
+    <t>0.19-0.22</t>
+  </si>
+  <si>
+    <t>0.23-0.29</t>
+  </si>
+  <si>
+    <t>0.30-0.39</t>
+  </si>
+  <si>
+    <t>0.40-0.49</t>
+  </si>
+  <si>
+    <t>0.50-0.69</t>
+  </si>
+  <si>
+    <t>0.70-0.89</t>
+  </si>
+  <si>
+    <t>0.90-0.99</t>
+  </si>
+  <si>
+    <t>1.00-1.49</t>
   </si>
 </sst>
 </file>
@@ -331,6 +355,15 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -338,15 +371,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -629,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H179"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
@@ -645,28 +669,28 @@
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="12"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
@@ -928,15 +952,15 @@
     </row>
     <row r="15" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3"/>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="12"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
@@ -1198,15 +1222,15 @@
     </row>
     <row r="26" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="12"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="9"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
@@ -1468,15 +1492,15 @@
     </row>
     <row r="37" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="12"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
@@ -1738,15 +1762,15 @@
     </row>
     <row r="48" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
-      <c r="B48" s="10" t="s">
+      <c r="B48" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
-      <c r="H48" s="12"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="9"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
@@ -2008,15 +2032,15 @@
     </row>
     <row r="59" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3"/>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C59" s="11"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="11"/>
-      <c r="F59" s="11"/>
-      <c r="G59" s="11"/>
-      <c r="H59" s="12"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="9"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
@@ -2278,15 +2302,15 @@
     </row>
     <row r="70" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3"/>
-      <c r="B70" s="10" t="s">
+      <c r="B70" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C70" s="11"/>
-      <c r="D70" s="11"/>
-      <c r="E70" s="11"/>
-      <c r="F70" s="11"/>
-      <c r="G70" s="11"/>
-      <c r="H70" s="12"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8"/>
+      <c r="H70" s="9"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
@@ -2548,15 +2572,15 @@
     </row>
     <row r="81" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3"/>
-      <c r="B81" s="10" t="s">
+      <c r="B81" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C81" s="11"/>
-      <c r="D81" s="11"/>
-      <c r="E81" s="11"/>
-      <c r="F81" s="11"/>
-      <c r="G81" s="11"/>
-      <c r="H81" s="12"/>
+      <c r="C81" s="8"/>
+      <c r="D81" s="8"/>
+      <c r="E81" s="8"/>
+      <c r="F81" s="8"/>
+      <c r="G81" s="8"/>
+      <c r="H81" s="9"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
@@ -2790,7 +2814,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>17</v>
       </c>
@@ -2816,8 +2840,1168 @@
         <v>56</v>
       </c>
     </row>
+    <row r="92" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A92" s="3"/>
+      <c r="B92" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C92" s="8"/>
+      <c r="D92" s="8"/>
+      <c r="E92" s="8"/>
+      <c r="F92" s="8"/>
+      <c r="G92" s="8"/>
+      <c r="H92" s="9"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="3"/>
+      <c r="B93" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C93" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D93" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F93" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H93" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B94"/>
+      <c r="C94"/>
+      <c r="D94"/>
+      <c r="E94"/>
+      <c r="F94"/>
+      <c r="G94"/>
+      <c r="H94"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B95"/>
+      <c r="C95"/>
+      <c r="D95"/>
+      <c r="E95"/>
+      <c r="F95"/>
+      <c r="G95"/>
+      <c r="H95"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B96"/>
+      <c r="C96"/>
+      <c r="D96"/>
+      <c r="E96"/>
+      <c r="F96"/>
+      <c r="G96"/>
+      <c r="H96"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B97"/>
+      <c r="C97"/>
+      <c r="D97"/>
+      <c r="E97"/>
+      <c r="F97"/>
+      <c r="G97"/>
+      <c r="H97"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B98"/>
+      <c r="C98"/>
+      <c r="D98"/>
+      <c r="E98"/>
+      <c r="F98"/>
+      <c r="G98"/>
+      <c r="H98"/>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B99"/>
+      <c r="C99"/>
+      <c r="D99"/>
+      <c r="E99"/>
+      <c r="F99"/>
+      <c r="G99"/>
+      <c r="H99"/>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B100"/>
+      <c r="C100"/>
+      <c r="D100"/>
+      <c r="E100"/>
+      <c r="F100"/>
+      <c r="G100"/>
+      <c r="H100"/>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B101"/>
+      <c r="C101"/>
+      <c r="D101"/>
+      <c r="E101"/>
+      <c r="F101"/>
+      <c r="G101"/>
+      <c r="H101"/>
+    </row>
+    <row r="102" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B102"/>
+      <c r="C102"/>
+      <c r="D102"/>
+      <c r="E102"/>
+      <c r="F102"/>
+      <c r="G102"/>
+      <c r="H102"/>
+    </row>
+    <row r="103" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="3"/>
+      <c r="B103" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C103" s="8"/>
+      <c r="D103" s="8"/>
+      <c r="E103" s="8"/>
+      <c r="F103" s="8"/>
+      <c r="G103" s="8"/>
+      <c r="H103" s="9"/>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" s="3"/>
+      <c r="B104" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D104" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E104" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F104" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G104" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H104" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B105"/>
+      <c r="C105"/>
+      <c r="D105"/>
+      <c r="E105"/>
+      <c r="F105"/>
+      <c r="G105"/>
+      <c r="H105"/>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B106"/>
+      <c r="C106"/>
+      <c r="D106"/>
+      <c r="E106"/>
+      <c r="F106"/>
+      <c r="G106"/>
+      <c r="H106"/>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B107"/>
+      <c r="C107"/>
+      <c r="D107"/>
+      <c r="E107"/>
+      <c r="F107"/>
+      <c r="G107"/>
+      <c r="H107"/>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B108"/>
+      <c r="C108"/>
+      <c r="D108"/>
+      <c r="E108"/>
+      <c r="F108"/>
+      <c r="G108"/>
+      <c r="H108"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B109"/>
+      <c r="C109"/>
+      <c r="D109"/>
+      <c r="E109"/>
+      <c r="F109"/>
+      <c r="G109"/>
+      <c r="H109"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B110"/>
+      <c r="C110"/>
+      <c r="D110"/>
+      <c r="E110"/>
+      <c r="F110"/>
+      <c r="G110"/>
+      <c r="H110"/>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B111"/>
+      <c r="C111"/>
+      <c r="D111"/>
+      <c r="E111"/>
+      <c r="F111"/>
+      <c r="G111"/>
+      <c r="H111"/>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B112"/>
+      <c r="C112"/>
+      <c r="D112"/>
+      <c r="E112"/>
+      <c r="F112"/>
+      <c r="G112"/>
+      <c r="H112"/>
+    </row>
+    <row r="113" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B113"/>
+      <c r="C113"/>
+      <c r="D113"/>
+      <c r="E113"/>
+      <c r="F113"/>
+      <c r="G113"/>
+      <c r="H113"/>
+    </row>
+    <row r="114" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A114" s="3"/>
+      <c r="B114" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C114" s="8"/>
+      <c r="D114" s="8"/>
+      <c r="E114" s="8"/>
+      <c r="F114" s="8"/>
+      <c r="G114" s="8"/>
+      <c r="H114" s="9"/>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" s="3"/>
+      <c r="B115" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C115" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D115" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E115" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F115" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G115" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H115" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B116"/>
+      <c r="C116"/>
+      <c r="D116"/>
+      <c r="E116"/>
+      <c r="F116"/>
+      <c r="G116"/>
+      <c r="H116"/>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B117"/>
+      <c r="C117"/>
+      <c r="D117"/>
+      <c r="E117"/>
+      <c r="F117"/>
+      <c r="G117"/>
+      <c r="H117"/>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B118"/>
+      <c r="C118"/>
+      <c r="D118"/>
+      <c r="E118"/>
+      <c r="F118"/>
+      <c r="G118"/>
+      <c r="H118"/>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B119"/>
+      <c r="C119"/>
+      <c r="D119"/>
+      <c r="E119"/>
+      <c r="F119"/>
+      <c r="G119"/>
+      <c r="H119"/>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B120"/>
+      <c r="C120"/>
+      <c r="D120"/>
+      <c r="E120"/>
+      <c r="F120"/>
+      <c r="G120"/>
+      <c r="H120"/>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B121"/>
+      <c r="C121"/>
+      <c r="D121"/>
+      <c r="E121"/>
+      <c r="F121"/>
+      <c r="G121"/>
+      <c r="H121"/>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B122"/>
+      <c r="C122"/>
+      <c r="D122"/>
+      <c r="E122"/>
+      <c r="F122"/>
+      <c r="G122"/>
+      <c r="H122"/>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A123" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B123"/>
+      <c r="C123"/>
+      <c r="D123"/>
+      <c r="E123"/>
+      <c r="F123"/>
+      <c r="G123"/>
+      <c r="H123"/>
+    </row>
+    <row r="124" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B124"/>
+      <c r="C124"/>
+      <c r="D124"/>
+      <c r="E124"/>
+      <c r="F124"/>
+      <c r="G124"/>
+      <c r="H124"/>
+    </row>
+    <row r="125" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A125" s="3"/>
+      <c r="B125" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C125" s="8"/>
+      <c r="D125" s="8"/>
+      <c r="E125" s="8"/>
+      <c r="F125" s="8"/>
+      <c r="G125" s="8"/>
+      <c r="H125" s="9"/>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="3"/>
+      <c r="B126" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F126" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G126" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B127"/>
+      <c r="C127"/>
+      <c r="D127"/>
+      <c r="E127"/>
+      <c r="F127"/>
+      <c r="G127"/>
+      <c r="H127"/>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B128"/>
+      <c r="C128"/>
+      <c r="D128"/>
+      <c r="E128"/>
+      <c r="F128"/>
+      <c r="G128"/>
+      <c r="H128"/>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B129"/>
+      <c r="C129"/>
+      <c r="D129"/>
+      <c r="E129"/>
+      <c r="F129"/>
+      <c r="G129"/>
+      <c r="H129"/>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B130"/>
+      <c r="C130"/>
+      <c r="D130"/>
+      <c r="E130"/>
+      <c r="F130"/>
+      <c r="G130"/>
+      <c r="H130"/>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B131"/>
+      <c r="C131"/>
+      <c r="D131"/>
+      <c r="E131"/>
+      <c r="F131"/>
+      <c r="G131"/>
+      <c r="H131"/>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B132"/>
+      <c r="C132"/>
+      <c r="D132"/>
+      <c r="E132"/>
+      <c r="F132"/>
+      <c r="G132"/>
+      <c r="H132"/>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B133"/>
+      <c r="C133"/>
+      <c r="D133"/>
+      <c r="E133"/>
+      <c r="F133"/>
+      <c r="G133"/>
+      <c r="H133"/>
+    </row>
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A134" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B134"/>
+      <c r="C134"/>
+      <c r="D134"/>
+      <c r="E134"/>
+      <c r="F134"/>
+      <c r="G134"/>
+      <c r="H134"/>
+    </row>
+    <row r="135" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B135"/>
+      <c r="C135"/>
+      <c r="D135"/>
+      <c r="E135"/>
+      <c r="F135"/>
+      <c r="G135"/>
+      <c r="H135"/>
+    </row>
+    <row r="136" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A136" s="3"/>
+      <c r="B136" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C136" s="8"/>
+      <c r="D136" s="8"/>
+      <c r="E136" s="8"/>
+      <c r="F136" s="8"/>
+      <c r="G136" s="8"/>
+      <c r="H136" s="9"/>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="3"/>
+      <c r="B137" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F137" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G137" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H137" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B138"/>
+      <c r="C138"/>
+      <c r="D138"/>
+      <c r="E138"/>
+      <c r="F138"/>
+      <c r="G138"/>
+      <c r="H138"/>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B139"/>
+      <c r="C139"/>
+      <c r="D139"/>
+      <c r="E139"/>
+      <c r="F139"/>
+      <c r="G139"/>
+      <c r="H139"/>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B140"/>
+      <c r="C140"/>
+      <c r="D140"/>
+      <c r="E140"/>
+      <c r="F140"/>
+      <c r="G140"/>
+      <c r="H140"/>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B141"/>
+      <c r="C141"/>
+      <c r="D141"/>
+      <c r="E141"/>
+      <c r="F141"/>
+      <c r="G141"/>
+      <c r="H141"/>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B142"/>
+      <c r="C142"/>
+      <c r="D142"/>
+      <c r="E142"/>
+      <c r="F142"/>
+      <c r="G142"/>
+      <c r="H142"/>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B143"/>
+      <c r="C143"/>
+      <c r="D143"/>
+      <c r="E143"/>
+      <c r="F143"/>
+      <c r="G143"/>
+      <c r="H143"/>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B144"/>
+      <c r="C144"/>
+      <c r="D144"/>
+      <c r="E144"/>
+      <c r="F144"/>
+      <c r="G144"/>
+      <c r="H144"/>
+    </row>
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A145" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B145"/>
+      <c r="C145"/>
+      <c r="D145"/>
+      <c r="E145"/>
+      <c r="F145"/>
+      <c r="G145"/>
+      <c r="H145"/>
+    </row>
+    <row r="146" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A146" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B146"/>
+      <c r="C146"/>
+      <c r="D146"/>
+      <c r="E146"/>
+      <c r="F146"/>
+      <c r="G146"/>
+      <c r="H146"/>
+    </row>
+    <row r="147" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A147" s="3"/>
+      <c r="B147" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C147" s="8"/>
+      <c r="D147" s="8"/>
+      <c r="E147" s="8"/>
+      <c r="F147" s="8"/>
+      <c r="G147" s="8"/>
+      <c r="H147" s="9"/>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="3"/>
+      <c r="B148" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C148" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E148" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F148" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G148" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H148" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B149"/>
+      <c r="C149"/>
+      <c r="D149"/>
+      <c r="E149"/>
+      <c r="F149"/>
+      <c r="G149"/>
+      <c r="H149"/>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B150"/>
+      <c r="C150"/>
+      <c r="D150"/>
+      <c r="E150"/>
+      <c r="F150"/>
+      <c r="G150"/>
+      <c r="H150"/>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B151"/>
+      <c r="C151"/>
+      <c r="D151"/>
+      <c r="E151"/>
+      <c r="F151"/>
+      <c r="G151"/>
+      <c r="H151"/>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B152"/>
+      <c r="C152"/>
+      <c r="D152"/>
+      <c r="E152"/>
+      <c r="F152"/>
+      <c r="G152"/>
+      <c r="H152"/>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B153"/>
+      <c r="C153"/>
+      <c r="D153"/>
+      <c r="E153"/>
+      <c r="F153"/>
+      <c r="G153"/>
+      <c r="H153"/>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B154"/>
+      <c r="C154"/>
+      <c r="D154"/>
+      <c r="E154"/>
+      <c r="F154"/>
+      <c r="G154"/>
+      <c r="H154"/>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B155"/>
+      <c r="C155"/>
+      <c r="D155"/>
+      <c r="E155"/>
+      <c r="F155"/>
+      <c r="G155"/>
+      <c r="H155"/>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B156"/>
+      <c r="C156"/>
+      <c r="D156"/>
+      <c r="E156"/>
+      <c r="F156"/>
+      <c r="G156"/>
+      <c r="H156"/>
+    </row>
+    <row r="157" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B157"/>
+      <c r="C157"/>
+      <c r="D157"/>
+      <c r="E157"/>
+      <c r="F157"/>
+      <c r="G157"/>
+      <c r="H157"/>
+    </row>
+    <row r="158" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A158" s="3"/>
+      <c r="B158" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C158" s="8"/>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="8"/>
+      <c r="H158" s="9"/>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="3"/>
+      <c r="B159" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E159" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G159" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H159" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B160"/>
+      <c r="C160"/>
+      <c r="D160"/>
+      <c r="E160"/>
+      <c r="F160"/>
+      <c r="G160"/>
+      <c r="H160"/>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B161"/>
+      <c r="C161"/>
+      <c r="D161"/>
+      <c r="E161"/>
+      <c r="F161"/>
+      <c r="G161"/>
+      <c r="H161"/>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B162"/>
+      <c r="C162"/>
+      <c r="D162"/>
+      <c r="E162"/>
+      <c r="F162"/>
+      <c r="G162"/>
+      <c r="H162"/>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B163"/>
+      <c r="C163"/>
+      <c r="D163"/>
+      <c r="E163"/>
+      <c r="F163"/>
+      <c r="G163"/>
+      <c r="H163"/>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B164"/>
+      <c r="C164"/>
+      <c r="D164"/>
+      <c r="E164"/>
+      <c r="F164"/>
+      <c r="G164"/>
+      <c r="H164"/>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B165"/>
+      <c r="C165"/>
+      <c r="D165"/>
+      <c r="E165"/>
+      <c r="F165"/>
+      <c r="G165"/>
+      <c r="H165"/>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A166" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B166"/>
+      <c r="C166"/>
+      <c r="D166"/>
+      <c r="E166"/>
+      <c r="F166"/>
+      <c r="G166"/>
+      <c r="H166"/>
+    </row>
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A167" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B167"/>
+      <c r="C167"/>
+      <c r="D167"/>
+      <c r="E167"/>
+      <c r="F167"/>
+      <c r="G167"/>
+      <c r="H167"/>
+    </row>
+    <row r="168" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A168" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B168"/>
+      <c r="C168"/>
+      <c r="D168"/>
+      <c r="E168"/>
+      <c r="F168"/>
+      <c r="G168"/>
+      <c r="H168"/>
+    </row>
+    <row r="169" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A169" s="3"/>
+      <c r="B169" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C169" s="8"/>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8"/>
+      <c r="F169" s="8"/>
+      <c r="G169" s="8"/>
+      <c r="H169" s="9"/>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" s="3"/>
+      <c r="B170" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E170" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F170" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G170" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H170" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B171"/>
+      <c r="C171"/>
+      <c r="D171"/>
+      <c r="E171"/>
+      <c r="F171"/>
+      <c r="G171"/>
+      <c r="H171"/>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B172"/>
+      <c r="C172"/>
+      <c r="D172"/>
+      <c r="E172"/>
+      <c r="F172"/>
+      <c r="G172"/>
+      <c r="H172"/>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B173"/>
+      <c r="C173"/>
+      <c r="D173"/>
+      <c r="E173"/>
+      <c r="F173"/>
+      <c r="G173"/>
+      <c r="H173"/>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B174"/>
+      <c r="C174"/>
+      <c r="D174"/>
+      <c r="E174"/>
+      <c r="F174"/>
+      <c r="G174"/>
+      <c r="H174"/>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B175"/>
+      <c r="C175"/>
+      <c r="D175"/>
+      <c r="E175"/>
+      <c r="F175"/>
+      <c r="G175"/>
+      <c r="H175"/>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B176"/>
+      <c r="C176"/>
+      <c r="D176"/>
+      <c r="E176"/>
+      <c r="F176"/>
+      <c r="G176"/>
+      <c r="H176"/>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B177"/>
+      <c r="C177"/>
+      <c r="D177"/>
+      <c r="E177"/>
+      <c r="F177"/>
+      <c r="G177"/>
+      <c r="H177"/>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B178"/>
+      <c r="C178"/>
+      <c r="D178"/>
+      <c r="E178"/>
+      <c r="F178"/>
+      <c r="G178"/>
+      <c r="H178"/>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B179"/>
+      <c r="C179"/>
+      <c r="D179"/>
+      <c r="E179"/>
+      <c r="F179"/>
+      <c r="G179"/>
+      <c r="H179"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="17">
+    <mergeCell ref="B147:H147"/>
+    <mergeCell ref="B158:H158"/>
+    <mergeCell ref="B169:H169"/>
+    <mergeCell ref="B92:H92"/>
+    <mergeCell ref="B103:H103"/>
+    <mergeCell ref="B114:H114"/>
+    <mergeCell ref="B125:H125"/>
+    <mergeCell ref="B136:H136"/>
     <mergeCell ref="B81:H81"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B37:H37"/>
@@ -2834,22 +4018,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F57AD1B-9C77-4ACE-A09B-12E013082B3A}">
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" ht="24" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="9"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2863,15 +4047,15 @@
     </row>
     <row r="3" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -3135,15 +4319,15 @@
     </row>
     <row r="14" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="12"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="9"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -3405,15 +4589,15 @@
     </row>
     <row r="25" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="12"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
@@ -3675,15 +4859,15 @@
     </row>
     <row r="36" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="12"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="9"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
@@ -3945,15 +5129,15 @@
     </row>
     <row r="47" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
-      <c r="B47" s="10" t="s">
+      <c r="B47" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="11"/>
-      <c r="H47" s="12"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
@@ -4215,15 +5399,15 @@
     </row>
     <row r="58" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
-      <c r="B58" s="10" t="s">
+      <c r="B58" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11"/>
-      <c r="G58" s="11"/>
-      <c r="H58" s="12"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="9"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
@@ -4485,15 +5669,15 @@
     </row>
     <row r="69" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3"/>
-      <c r="B69" s="10" t="s">
+      <c r="B69" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C69" s="11"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="11"/>
-      <c r="G69" s="11"/>
-      <c r="H69" s="12"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="8"/>
+      <c r="F69" s="8"/>
+      <c r="G69" s="8"/>
+      <c r="H69" s="9"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
@@ -4755,15 +5939,15 @@
     </row>
     <row r="80" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3"/>
-      <c r="B80" s="10" t="s">
+      <c r="B80" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C80" s="11"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="11"/>
-      <c r="G80" s="11"/>
-      <c r="H80" s="12"/>
+      <c r="C80" s="8"/>
+      <c r="D80" s="8"/>
+      <c r="E80" s="8"/>
+      <c r="F80" s="8"/>
+      <c r="G80" s="8"/>
+      <c r="H80" s="9"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
@@ -4997,7 +6181,7 @@
         <v>50.4</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>17</v>
       </c>
@@ -5023,8 +6207,664 @@
         <v>44.8</v>
       </c>
     </row>
+    <row r="91" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="3"/>
+      <c r="B91" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C91" s="8"/>
+      <c r="D91" s="8"/>
+      <c r="E91" s="8"/>
+      <c r="F91" s="8"/>
+      <c r="G91" s="8"/>
+      <c r="H91" s="9"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="3"/>
+      <c r="B92" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F92" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H92" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="3"/>
+      <c r="B102" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C102" s="8"/>
+      <c r="D102" s="8"/>
+      <c r="E102" s="8"/>
+      <c r="F102" s="8"/>
+      <c r="G102" s="8"/>
+      <c r="H102" s="9"/>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" s="3"/>
+      <c r="B103" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D103" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F103" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G103" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H103" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A113" s="3"/>
+      <c r="B113" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C113" s="8"/>
+      <c r="D113" s="8"/>
+      <c r="E113" s="8"/>
+      <c r="F113" s="8"/>
+      <c r="G113" s="8"/>
+      <c r="H113" s="9"/>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A114" s="3"/>
+      <c r="B114" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C114" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F114" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G114" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A118" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A119" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A120" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A121" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A124" s="3"/>
+      <c r="B124" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C124" s="8"/>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
+      <c r="G124" s="8"/>
+      <c r="H124" s="9"/>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A125" s="3"/>
+      <c r="B125" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F125" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G125" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H125" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A126" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A127" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A128" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A129" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A130" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A131" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A132" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A133" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="134" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="135" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A135" s="3"/>
+      <c r="B135" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C135" s="8"/>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+      <c r="G135" s="8"/>
+      <c r="H135" s="9"/>
+    </row>
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A136" s="3"/>
+      <c r="B136" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F136" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G136" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H136" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A137" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A138" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A139" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A141" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A142" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A143" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A144" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="145" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A146" s="3"/>
+      <c r="B146" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C146" s="8"/>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="8"/>
+      <c r="H146" s="9"/>
+    </row>
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A147" s="3"/>
+      <c r="B147" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C147" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E147" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F147" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G147" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H147" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A148" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A149" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A150" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A151" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A152" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A156" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A157" s="3"/>
+      <c r="B157" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C157" s="8"/>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8"/>
+      <c r="F157" s="8"/>
+      <c r="G157" s="8"/>
+      <c r="H157" s="9"/>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" s="3"/>
+      <c r="B158" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H158" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A161" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A162" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A163" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A164" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A165" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A166" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A168" s="3"/>
+      <c r="B168" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="8"/>
+      <c r="H168" s="9"/>
+    </row>
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A169" s="3"/>
+      <c r="B169" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D169" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E169" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F169" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G169" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H169" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A170" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A171" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A172" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A173" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A174" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A175" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A176" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="17">
+    <mergeCell ref="B146:H146"/>
+    <mergeCell ref="B157:H157"/>
+    <mergeCell ref="B168:H168"/>
+    <mergeCell ref="B91:H91"/>
+    <mergeCell ref="B102:H102"/>
+    <mergeCell ref="B113:H113"/>
+    <mergeCell ref="B124:H124"/>
+    <mergeCell ref="B135:H135"/>
     <mergeCell ref="B80:H80"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B36:H36"/>

</xml_diff>